<commit_message>
Dashboard update — 03 Jul 2026
</commit_message>
<xml_diff>
--- a/PIC_2026_Tracker.xlsx
+++ b/PIC_2026_Tracker.xlsx
@@ -2345,7 +2345,7 @@
       </c>
       <c r="J20" s="140" t="inlineStr">
         <is>
-          <t>Partial — $10 SGM still pending</t>
+          <t>$20 cash bet lost; $10 SGM on row 21 (settled loss)</t>
         </is>
       </c>
     </row>
@@ -2374,23 +2374,21 @@
       <c r="F21" s="151" t="n">
         <v>10</v>
       </c>
-      <c r="G21" s="149" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
+      <c r="G21" s="149" t="n">
+        <v>0</v>
       </c>
       <c r="H21" s="149" t="inlineStr">
         <is>
-          <t>Pending</t>
+          <t>Loss</t>
         </is>
       </c>
       <c r="I21" s="153">
-        <f>IF(G20="",I19+C20,I19+C20+G20)</f>
-        <v/>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>Pot. $117.50 | U178.5 pts, GEE H2H, Weitering/Dangerfield/De Koning 10+ disp, McGovern/Mannagh/S.Neale/Kemp 1+ goal</t>
+        <f>IF(G21="",I20+C21,I20+C21+G21)</f>
+        <v/>
+      </c>
+      <c r="J21" s="88" t="inlineStr">
+        <is>
+          <t>SGM lost — Carlton v Geelong Cats 29 May</t>
         </is>
       </c>
     </row>
@@ -2408,17 +2406,27 @@
       <c r="C22" s="143" t="n">
         <v>0</v>
       </c>
-      <c r="D22" s="135" t="n"/>
+      <c r="D22" s="135" t="inlineStr">
+        <is>
+          <t>Eagle Farm Race 6 — Brave Monarch</t>
+        </is>
+      </c>
       <c r="E22" s="136" t="n">
-        <v>30</v>
+        <v>3.9</v>
       </c>
       <c r="F22" s="143" t="n">
         <v>30</v>
       </c>
-      <c r="G22" s="137" t="n"/>
-      <c r="H22" s="154" t="n"/>
+      <c r="G22" s="137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="154" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="I22" s="144">
-        <f>IF(G21="",I20+C21,I20+C21+G21)</f>
+        <f>IF(G22="",I21+C22,I21+C22+G22)</f>
         <v/>
       </c>
       <c r="J22" s="140" t="n"/>
@@ -2437,17 +2445,25 @@
       <c r="C23" s="145" t="n">
         <v>0</v>
       </c>
-      <c r="D23" s="135" t="n"/>
-      <c r="E23" s="136" t="n">
-        <v>30</v>
-      </c>
+      <c r="D23" s="135" t="inlineStr">
+        <is>
+          <t>Sports Multi — Crusaders, Broncos, Panthers, Bulldogs, QLD State of Origin</t>
+        </is>
+      </c>
+      <c r="E23" s="136" t="n"/>
       <c r="F23" s="145" t="n">
         <v>30</v>
       </c>
-      <c r="G23" s="137" t="n"/>
-      <c r="H23" s="154" t="n"/>
+      <c r="G23" s="137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="154" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="I23" s="146">
-        <f>IF(G22="",I21+C22,I21+C22+G22)</f>
+        <f>IF(G23="",I22+C23,I22+C23+G23)</f>
         <v/>
       </c>
       <c r="J23" s="140" t="n"/>
@@ -2466,17 +2482,25 @@
       <c r="C24" s="134" t="n">
         <v>0</v>
       </c>
-      <c r="D24" s="135" t="n"/>
-      <c r="E24" s="136" t="n">
-        <v>30</v>
-      </c>
+      <c r="D24" s="135" t="inlineStr">
+        <is>
+          <t>Various Horses</t>
+        </is>
+      </c>
+      <c r="E24" s="136" t="n"/>
       <c r="F24" s="134" t="n">
         <v>30</v>
       </c>
-      <c r="G24" s="137" t="n"/>
-      <c r="H24" s="154" t="n"/>
+      <c r="G24" s="137" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="154" t="inlineStr">
+        <is>
+          <t>Loss</t>
+        </is>
+      </c>
       <c r="I24" s="139">
-        <f>IF(G23="",I22+C23,I22+C23+G23)</f>
+        <f>IF(G24="",I23+C24,I23+C24+G24)</f>
         <v/>
       </c>
       <c r="J24" s="140" t="n"/>
@@ -2495,17 +2519,27 @@
       <c r="C25" s="141" t="n">
         <v>0</v>
       </c>
-      <c r="D25" s="135" t="n"/>
+      <c r="D25" s="135" t="inlineStr">
+        <is>
+          <t>Flemington Race 3 — Vegas Jack (Place)</t>
+        </is>
+      </c>
       <c r="E25" s="136" t="n">
-        <v>30</v>
+        <v>2.88</v>
       </c>
       <c r="F25" s="141" t="n">
         <v>30</v>
       </c>
-      <c r="G25" s="137" t="n"/>
-      <c r="H25" s="154" t="n"/>
+      <c r="G25" s="137" t="n">
+        <v>86.40000000000001</v>
+      </c>
+      <c r="H25" s="154" t="inlineStr">
+        <is>
+          <t>Win</t>
+        </is>
+      </c>
       <c r="I25" s="142">
-        <f>IF(G24="",I23+C24,I23+C24+G24)</f>
+        <f>IF(G25="",I24+C25,I24+C25+G25)</f>
         <v/>
       </c>
       <c r="J25" s="140" t="n"/>
@@ -2534,10 +2568,14 @@
       <c r="G26" s="137" t="n"/>
       <c r="H26" s="154" t="n"/>
       <c r="I26" s="144">
-        <f>IF(G25="",I24+C25,I24+C25+G25)</f>
-        <v/>
-      </c>
-      <c r="J26" s="140" t="n"/>
+        <f>IF(G26="",I25+C26,I25+C26+G26)</f>
+        <v/>
+      </c>
+      <c r="J26" s="140" t="inlineStr">
+        <is>
+          <t>BET OUTSTANDING</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="19.5" customHeight="1" s="89">
       <c r="A27" s="120" t="inlineStr">
@@ -2563,7 +2601,7 @@
       <c r="G27" s="137" t="n"/>
       <c r="H27" s="154" t="n"/>
       <c r="I27" s="146">
-        <f>IF(G26="",I25+C26,I25+C26+G26)</f>
+        <f>IF(G27="",I26+C27,I26+C27+G27)</f>
         <v/>
       </c>
       <c r="J27" s="140" t="n"/>
@@ -2592,7 +2630,7 @@
       <c r="G28" s="137" t="n"/>
       <c r="H28" s="154" t="n"/>
       <c r="I28" s="139">
-        <f>IF(G27="",I26+C27,I26+C27+G27)</f>
+        <f>IF(G28="",I27+C28,I27+C28+G28)</f>
         <v/>
       </c>
       <c r="J28" s="140" t="n"/>
@@ -2621,7 +2659,7 @@
       <c r="G29" s="137" t="n"/>
       <c r="H29" s="154" t="n"/>
       <c r="I29" s="142">
-        <f>IF(G28="",I27+C28,I27+C28+G28)</f>
+        <f>IF(G29="",I28+C29,I28+C29+G29)</f>
         <v/>
       </c>
       <c r="J29" s="140" t="n"/>
@@ -2650,7 +2688,7 @@
       <c r="G30" s="137" t="n"/>
       <c r="H30" s="154" t="n"/>
       <c r="I30" s="144">
-        <f>IF(G29="",I28+C29,I28+C29+G29)</f>
+        <f>IF(G30="",I29+C30,I29+C30+G30)</f>
         <v/>
       </c>
       <c r="J30" s="140" t="n"/>
@@ -2679,7 +2717,7 @@
       <c r="G31" s="137" t="n"/>
       <c r="H31" s="154" t="n"/>
       <c r="I31" s="146">
-        <f>IF(G30="",I29+C30,I29+C30+G30)</f>
+        <f>IF(G31="",I30+C31,I30+C31+G31)</f>
         <v/>
       </c>
       <c r="J31" s="140" t="n"/>
@@ -2708,7 +2746,7 @@
       <c r="G32" s="137" t="n"/>
       <c r="H32" s="154" t="n"/>
       <c r="I32" s="139">
-        <f>IF(G31="",I30+C31,I30+C31+G31)</f>
+        <f>IF(G32="",I31+C32,I31+C32+G32)</f>
         <v/>
       </c>
       <c r="J32" s="140" t="n"/>
@@ -2737,7 +2775,7 @@
       <c r="G33" s="137" t="n"/>
       <c r="H33" s="154" t="n"/>
       <c r="I33" s="142">
-        <f>IF(G32="",I31+C32,I31+C32+G32)</f>
+        <f>IF(G33="",I32+C33,I32+C33+G33)</f>
         <v/>
       </c>
       <c r="J33" s="140" t="n"/>
@@ -2766,7 +2804,7 @@
       <c r="G34" s="137" t="n"/>
       <c r="H34" s="154" t="n"/>
       <c r="I34" s="144">
-        <f>IF(G33="",I32+C33,I32+C33+G33)</f>
+        <f>IF(G34="",I33+C34,I33+C34+G34)</f>
         <v/>
       </c>
       <c r="J34" s="140" t="n"/>
@@ -2795,7 +2833,7 @@
       <c r="G35" s="137" t="n"/>
       <c r="H35" s="154" t="n"/>
       <c r="I35" s="146">
-        <f>IF(G34="",I33+C34,I33+C34+G34)</f>
+        <f>IF(G35="",I34+C35,I34+C35+G35)</f>
         <v/>
       </c>
       <c r="J35" s="140" t="n"/>
@@ -2824,7 +2862,7 @@
       <c r="G36" s="137" t="n"/>
       <c r="H36" s="154" t="n"/>
       <c r="I36" s="139">
-        <f>IF(G35="",I34+C35,I34+C35+G35)</f>
+        <f>IF(G36="",I35+C36,I35+C36+G36)</f>
         <v/>
       </c>
       <c r="J36" s="140" t="n"/>
@@ -2853,7 +2891,7 @@
       <c r="G37" s="137" t="n"/>
       <c r="H37" s="154" t="n"/>
       <c r="I37" s="142">
-        <f>IF(G36="",I35+C36,I35+C36+G36)</f>
+        <f>IF(G37="",I36+C37,I36+C37+G37)</f>
         <v/>
       </c>
       <c r="J37" s="140" t="n"/>
@@ -2882,7 +2920,7 @@
       <c r="G38" s="137" t="n"/>
       <c r="H38" s="154" t="n"/>
       <c r="I38" s="144">
-        <f>IF(G37="",I36+C37,I36+C37+G37)</f>
+        <f>IF(G38="",I37+C38,I37+C38+G38)</f>
         <v/>
       </c>
       <c r="J38" s="140" t="n"/>
@@ -2911,7 +2949,7 @@
       <c r="G39" s="137" t="n"/>
       <c r="H39" s="154" t="n"/>
       <c r="I39" s="146">
-        <f>IF(G38="",I37+C38,I37+C38+G38)</f>
+        <f>IF(G39="",I38+C39,I38+C39+G39)</f>
         <v/>
       </c>
       <c r="J39" s="140" t="n"/>
@@ -2940,7 +2978,7 @@
       <c r="G40" s="137" t="n"/>
       <c r="H40" s="154" t="n"/>
       <c r="I40" s="139">
-        <f>IF(G39="",I38+C39,I38+C39+G39)</f>
+        <f>IF(G40="",I39+C40,I39+C40+G40)</f>
         <v/>
       </c>
       <c r="J40" s="140" t="n"/>
@@ -2969,7 +3007,7 @@
       <c r="G41" s="137" t="n"/>
       <c r="H41" s="154" t="n"/>
       <c r="I41" s="142">
-        <f>IF(G40="",I39+C40,I39+C40+G40)</f>
+        <f>IF(G41="",I40+C41,I40+C41+G41)</f>
         <v/>
       </c>
       <c r="J41" s="140" t="n"/>
@@ -2998,7 +3036,7 @@
       <c r="G42" s="137" t="n"/>
       <c r="H42" s="154" t="n"/>
       <c r="I42" s="144">
-        <f>IF(G41="",I40+C41,I40+C41+G41)</f>
+        <f>IF(G42="",I41+C42,I41+C42+G42)</f>
         <v/>
       </c>
       <c r="J42" s="140" t="n"/>
@@ -3027,7 +3065,7 @@
       <c r="G43" s="137" t="n"/>
       <c r="H43" s="154" t="n"/>
       <c r="I43" s="146">
-        <f>IF(G42="",I41+C42,I41+C42+G42)</f>
+        <f>IF(G43="",I42+C43,I42+C43+G43)</f>
         <v/>
       </c>
       <c r="J43" s="140" t="n"/>
@@ -3056,7 +3094,7 @@
       <c r="G44" s="137" t="n"/>
       <c r="H44" s="154" t="n"/>
       <c r="I44" s="139">
-        <f>IF(G43="",I42+C43,I42+C43+G43)</f>
+        <f>IF(G44="",I43+C44,I43+C44+G44)</f>
         <v/>
       </c>
       <c r="J44" s="140" t="n"/>
@@ -3085,7 +3123,7 @@
       <c r="G45" s="137" t="n"/>
       <c r="H45" s="154" t="n"/>
       <c r="I45" s="142">
-        <f>IF(G44="",I43+C44,I43+C44+G44)</f>
+        <f>IF(G45="",I44+C45,I44+C45+G45)</f>
         <v/>
       </c>
       <c r="J45" s="140" t="n"/>
@@ -3114,7 +3152,7 @@
       <c r="G46" s="137" t="n"/>
       <c r="H46" s="154" t="n"/>
       <c r="I46" s="144">
-        <f>IF(G45="",I44+C45,I44+C45+G45)</f>
+        <f>IF(G46="",I45+C46,I45+C46+G46)</f>
         <v/>
       </c>
       <c r="J46" s="140" t="n"/>
@@ -3143,7 +3181,7 @@
       <c r="G47" s="137" t="n"/>
       <c r="H47" s="154" t="n"/>
       <c r="I47" s="146">
-        <f>IF(G46="",I45+C46,I45+C46+G46)</f>
+        <f>IF(G47="",I46+C47,I46+C47+G47)</f>
         <v/>
       </c>
       <c r="J47" s="140" t="n"/>
@@ -3172,7 +3210,7 @@
       <c r="G48" s="137" t="n"/>
       <c r="H48" s="154" t="n"/>
       <c r="I48" s="139">
-        <f>IF(G47="",I46+C47,I46+C47+G47)</f>
+        <f>IF(G48="",I47+C48,I47+C48+G48)</f>
         <v/>
       </c>
       <c r="J48" s="140" t="n"/>
@@ -3201,7 +3239,7 @@
       <c r="G49" s="137" t="n"/>
       <c r="H49" s="154" t="n"/>
       <c r="I49" s="142">
-        <f>IF(G48="",I47+C48,I47+C48+G48)</f>
+        <f>IF(G49="",I48+C49,I48+C49+G49)</f>
         <v/>
       </c>
       <c r="J49" s="140" t="n"/>
@@ -3230,7 +3268,7 @@
       <c r="G50" s="137" t="n"/>
       <c r="H50" s="154" t="n"/>
       <c r="I50" s="144">
-        <f>IF(G49="",I48+C49,I48+C49+G49)</f>
+        <f>IF(G50="",I49+C50,I49+C50+G50)</f>
         <v/>
       </c>
       <c r="J50" s="140" t="n"/>
@@ -3259,7 +3297,7 @@
       <c r="G51" s="137" t="n"/>
       <c r="H51" s="154" t="n"/>
       <c r="I51" s="146">
-        <f>IF(G50="",I49+C50,I49+C50+G50)</f>
+        <f>IF(G51="",I50+C51,I50+C51+G51)</f>
         <v/>
       </c>
       <c r="J51" s="140" t="n"/>

</xml_diff>